<commit_message>
:duck: save mtd & LBM memberships in scrip 5 to charge them in script 6
</commit_message>
<xml_diff>
--- a/data/derived_data/6_NMI_CCA/Dataset_1/CCA_NULL_ITS_D1.xlsx
+++ b/data/derived_data/6_NMI_CCA/Dataset_1/CCA_NULL_ITS_D1.xlsx
@@ -410,10 +410,10 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>1.13382485197001</v>
+        <v>0.858202069228945</v>
       </c>
       <c r="D2" t="n">
-        <v>12.4638833895768</v>
+        <v>11.8823014191423</v>
       </c>
       <c r="E2" t="n">
         <v>0.001</v>
@@ -427,10 +427,10 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.707668925250851</v>
+        <v>0.538286356209151</v>
       </c>
       <c r="D3" t="n">
-        <v>4.67126584590073</v>
+        <v>4.50941525971249</v>
       </c>
       <c r="E3" t="n">
         <v>0.001</v>
@@ -444,10 +444,10 @@
         <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>1.8335220342951</v>
+        <v>1.43811759260887</v>
       </c>
       <c r="D4" t="n">
-        <v>9.84370487355589</v>
+        <v>9.76752330208493</v>
       </c>
       <c r="E4" t="n">
         <v>0.001</v>
@@ -461,10 +461,10 @@
         <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>1.12585310904425</v>
+        <v>0.899831236399721</v>
       </c>
       <c r="D5" t="n">
-        <v>14.5777036729003</v>
+        <v>14.7520088430891</v>
       </c>
       <c r="E5" t="n">
         <v>0.001</v>
@@ -478,10 +478,10 @@
         <v>14</v>
       </c>
       <c r="C6" t="n">
-        <v>0.699697182325084</v>
+        <v>0.579915523379922</v>
       </c>
       <c r="D6" t="n">
-        <v>6.11350810605897</v>
+        <v>6.4136198373875</v>
       </c>
       <c r="E6" t="n">
         <v>0.001</v>

</xml_diff>